<commit_message>
Stamp TIME at mid-exposure and average pointing over each exposure
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level1_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level1_nirda.xlsx
@@ -643,7 +643,6 @@
           <t>True</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -673,7 +672,6 @@
           <t>NEXTEND</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>2</t>
@@ -691,7 +689,6 @@
           <t>SIMDATA</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>False</t>
@@ -709,7 +706,6 @@
           <t>SCIDATA</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>True</t>
@@ -793,7 +789,6 @@
           <t>CREATOR</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Pandora MOC</t>
@@ -811,7 +806,6 @@
           <t>CRSOFTV</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>v3.06</t>
@@ -829,7 +823,6 @@
           <t>COMPTYPE</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>1</t>
@@ -847,7 +840,6 @@
           <t>TRANSID</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>0</t>
@@ -865,7 +857,6 @@
           <t>TARG_ID</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>KELT-9b</t>
@@ -883,7 +874,6 @@
           <t>FILENAME</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>/sssp/data/2026/08/15/2026-08-15__06-44-18_InfImg_KELT-9b_d0080x0250x3096_b1_e01_i387_g02_d16_r04.sp</t>
@@ -901,7 +891,6 @@
           <t>BINSIZE</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>1</t>
@@ -919,7 +908,6 @@
           <t>BITDEPTH</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>32</t>
@@ -937,7 +925,6 @@
           <t>BITSPIX</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>16</t>
@@ -955,7 +942,6 @@
           <t>ROISTRTX</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>1737</t>
@@ -973,7 +959,6 @@
           <t>ROISTRTY</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>962</t>
@@ -991,7 +976,6 @@
           <t>ROISTRTZ</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>0</t>
@@ -1009,7 +993,6 @@
           <t>ROISIZEX</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>80</t>
@@ -1027,7 +1010,6 @@
           <t>ROISIZEY</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>250</t>
@@ -1045,7 +1027,6 @@
           <t>ROISIZEZ</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>774</t>
@@ -1063,7 +1044,6 @@
           <t>RICEX</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>5</t>
@@ -1081,7 +1061,6 @@
           <t>RICEY</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>28</t>
@@ -1099,7 +1078,6 @@
           <t>CORSTIME</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>840091495</t>
@@ -1117,7 +1095,6 @@
           <t>FINETIME</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>832000000</t>
@@ -1135,7 +1112,6 @@
           <t>COMMAND</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>10</t>
@@ -1153,7 +1129,6 @@
           <t>CONFIG1</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>53251</t>
@@ -1171,7 +1146,6 @@
           <t>CONFIG2</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>0</t>
@@ -1189,7 +1163,6 @@
           <t>CONFIG3</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>0</t>
@@ -1207,7 +1180,6 @@
           <t>GAINREG</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>37002</t>
@@ -1225,7 +1197,6 @@
           <t>RESETS1</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>259</t>
@@ -1243,7 +1214,6 @@
           <t>RESETS2</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>1</t>
@@ -1261,7 +1231,6 @@
           <t>DROPS1</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>1</t>
@@ -1279,7 +1248,6 @@
           <t>DROPS2</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>16</t>
@@ -1297,7 +1265,6 @@
           <t>DROPS3</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>0</t>
@@ -1315,7 +1282,6 @@
           <t>READS</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>4</t>
@@ -1333,7 +1299,6 @@
           <t>GRPS</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>2</t>
@@ -1351,7 +1316,6 @@
           <t>INTEGRTS</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>387</t>
@@ -1369,7 +1333,6 @@
           <t>EXPOSRES</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>1</t>
@@ -1387,7 +1350,6 @@
           <t>ENDDELAY</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>0</t>
@@ -1405,7 +1367,6 @@
           <t>RSTSINC</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>0</t>
@@ -1423,7 +1384,6 @@
           <t>DRPSINC</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>0</t>
@@ -1441,7 +1401,6 @@
           <t>FRMSTOT</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>10320</t>
@@ -1459,7 +1418,6 @@
           <t>FRMSEXP</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>3096</t>
@@ -1477,7 +1435,6 @@
           <t>FRMSACQ</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>3096</t>
@@ -1495,7 +1452,6 @@
           <t>GRPSAVGD</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>1</t>
@@ -1513,7 +1469,6 @@
           <t>PAMPGAIN</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>5.65685</t>
@@ -1531,7 +1486,6 @@
           <t>FRMTIME</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>231</t>
@@ -1549,7 +1503,6 @@
           <t>TSIDECAR</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>3.3816466331481934</t>
@@ -1567,7 +1520,6 @@
           <t>TCOMPRJT</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>278.990966796875</t>
@@ -1585,7 +1537,6 @@
           <t>TCLDTIP1</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>131.50372314453125</t>
@@ -1603,7 +1554,6 @@
           <t>TCLDTIP2</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>120.03438568115234</t>
@@ -1621,7 +1571,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>EOXEFNVBENVBENVB</t>
@@ -1639,7 +1588,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>0</t>
@@ -1657,13 +1605,11 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1671,13 +1617,11 @@
           <t>PFSOFTV</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>0.6.0</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1685,13 +1629,11 @@
           <t>PRSOFTV</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>2.9.1</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1699,13 +1641,11 @@
           <t>PFCLASS</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>NIRDALevel1HDUList</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1713,7 +1653,6 @@
           <t>PFTIME</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>2026-09-09T19:45:55.608</t>
@@ -1833,13 +1772,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1847,13 +1784,11 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>250</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1861,13 +1796,11 @@
           <t>NAXIS3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1875,7 +1808,6 @@
           <t>NAXIS4</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>2</t>
@@ -1893,7 +1825,6 @@
           <t>NAXIS5</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>387</t>
@@ -1911,7 +1842,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>0</t>
@@ -1929,7 +1859,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>1</t>
@@ -1969,7 +1898,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>iX5ajU2SiU2YiU2Y</t>
@@ -1987,7 +1915,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>1317043718</t>
@@ -2005,20 +1932,13 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>ct</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="16"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2030,7 +1950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2127,13 +2047,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2141,13 +2059,11 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2155,13 +2071,11 @@
           <t>NAXIS3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2169,7 +2083,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>0</t>
@@ -2187,7 +2100,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -2205,7 +2117,6 @@
           <t>FRAME</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>JD</t>
@@ -2242,34 +2153,49 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CHECKSUM</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>TIMEPIXR</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ZLiAaJi5UJiAZJi5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-09-09T15:46:04</t>
+          <t>TIME is the middle of each exposure</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>CHECKSUM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ZLiAaJi5UJiAZJi5</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>HDU checksum updated 2026-09-09T15:46:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>4049659845</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>data unit checksum updated 2026-09-09T15:46:04</t>
         </is>
@@ -2383,13 +2309,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2397,13 +2321,11 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2411,13 +2333,11 @@
           <t>NAXIS3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2425,7 +2345,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>0</t>
@@ -2443,7 +2362,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -2461,7 +2379,6 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>second</t>
@@ -2501,7 +2418,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>6S3a9R3U6R3Z6R3Z</t>
@@ -2519,7 +2435,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>379881537</t>
@@ -2639,13 +2554,11 @@
           <t>NAXIS1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2653,13 +2566,11 @@
           <t>NAXIS2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2667,13 +2578,11 @@
           <t>NAXIS3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>387</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2681,7 +2590,6 @@
           <t>PCOUNT</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>0</t>
@@ -2699,7 +2607,6 @@
           <t>GCOUNT</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>1</t>
@@ -2739,7 +2646,6 @@
           <t>CHECKSUM</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>oT5aqR3UoR3aoR3U</t>
@@ -2757,7 +2663,6 @@
           <t>DATASUM</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>149382</t>

</xml_diff>

<commit_message>
Add UTC metadata and document FITS timestamp conventions
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level1_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level1_nirda.xlsx
@@ -2030,7 +2030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2272,6 +2272,28 @@
       <c r="D13" t="inlineStr">
         <is>
           <t>data unit checksum updated 2026-09-09T15:46:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TIMESYS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Time scale</t>
         </is>
       </c>
     </row>

</xml_diff>